<commit_message>
estimate given to laganshil krishak samuha badri dhakal
</commit_message>
<xml_diff>
--- a/बजेट माग estimate/lagansil krishak samuha.xlsx
+++ b/बजेट माग estimate/lagansil krishak samuha.xlsx
@@ -1,10 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
-  <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4BC52F6-C133-4B16-AAC9-3969749A9F55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8424"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="estimate" sheetId="6" r:id="rId1"/>
@@ -22,9 +23,9 @@
     <definedName name="description_6">[2]Abstract!$B$172</definedName>
     <definedName name="description_783">[3]Abstract!$B$301</definedName>
     <definedName name="description_8">[4]Abstract!$B$174</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">estimate!$A$1:$L$30</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">estimate!$A$1:$L$32</definedName>
   </definedNames>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="85">
   <si>
     <t>Government of Nepal</t>
   </si>
@@ -72,15 +73,9 @@
     <t>Shankhu, Kathmandu</t>
   </si>
   <si>
-    <t>Estimate Sheet</t>
-  </si>
-  <si>
     <t xml:space="preserve">Project:- </t>
   </si>
   <si>
-    <t>F.Y.:-081/82</t>
-  </si>
-  <si>
     <t>Location:- Shankharapur Municipality- 1</t>
   </si>
   <si>
@@ -138,18 +133,6 @@
     <t>md.</t>
   </si>
   <si>
-    <t>Skilled   mason</t>
-  </si>
-  <si>
-    <t>Unskilled mason</t>
-  </si>
-  <si>
-    <t>Fabrication of chain link mesh size 3"x3" 10 gauge</t>
-  </si>
-  <si>
-    <t>unit wt.</t>
-  </si>
-  <si>
     <t>page 6 sn.22</t>
   </si>
   <si>
@@ -160,9 +143,6 @@
   </si>
   <si>
     <t>district rate ktm</t>
-  </si>
-  <si>
-    <t>Date: 2082/01/25</t>
   </si>
   <si>
     <t>lh=cfO{=sf9]tf/ -jf/ j]8 jfo/_ nufpg]</t>
@@ -199,9 +179,6 @@
     <t>no.</t>
   </si>
   <si>
-    <t>vertical pole (40x40x2)</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">%) dL=dL= </t>
     </r>
@@ -568,19 +545,64 @@
   </si>
   <si>
     <t>hDdf b/ /]6</t>
+  </si>
+  <si>
+    <t>F.Y.:-2082/2083</t>
+  </si>
+  <si>
+    <t>Total Estimated</t>
+  </si>
+  <si>
+    <t>Budget allocated</t>
+  </si>
+  <si>
+    <t>Municipal payment</t>
+  </si>
+  <si>
+    <t>User Contribution</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contingencies </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maintanince </t>
+  </si>
+  <si>
+    <t>Unit wt. (Kg/m)</t>
+  </si>
+  <si>
+    <t>Length (m)</t>
+  </si>
+  <si>
+    <t>-Fabrication of chain link mesh size 3"x3" 10 gauge</t>
+  </si>
+  <si>
+    <t>-Skilled   mason</t>
+  </si>
+  <si>
+    <t>-Unskilled mason</t>
+  </si>
+  <si>
+    <t>-Vertical pole (40x40x2)</t>
+  </si>
+  <si>
+    <t>Estimated Sheet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date:                </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
-    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="_(* #,##0.0_);_(* \(#,##0.0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="25">
+  <fonts count="26">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -718,6 +740,13 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -733,42 +762,12 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="14">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="hair">
-        <color auto="1"/>
-      </top>
-      <bottom style="hair">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="hair">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -790,66 +789,6 @@
       </top>
       <bottom style="thin">
         <color theme="4" tint="0.39997558519241921"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="hair">
-        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
@@ -936,91 +875,243 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="86">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="1" fontId="14" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="14" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="14" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="14" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="15" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="2" fontId="14" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="25" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="5" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="166" fontId="3" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="11" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1028,91 +1119,37 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="1" fontId="14" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="14" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="14" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="14" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="15" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="2" fontId="14" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Comma 2" xfId="2"/>
+    <cellStyle name="Comma 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1129,7 +1166,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Datasheet"/>
@@ -1193,7 +1230,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Datasheet"/>
@@ -1302,7 +1339,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink3.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Datasheet"/>
@@ -1373,7 +1410,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink4.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Datasheet"/>
@@ -1705,740 +1742,834 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O38"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:O45"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="3.6640625" customWidth="1"/>
-    <col min="2" max="2" width="9.6640625" customWidth="1"/>
-    <col min="3" max="3" width="32.21875" customWidth="1"/>
-    <col min="4" max="4" width="9.88671875" customWidth="1"/>
-    <col min="5" max="5" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.88671875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.109375" customWidth="1"/>
-    <col min="10" max="10" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.33203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="14.88671875" customWidth="1"/>
+    <col min="1" max="1" width="3.7109375" customWidth="1"/>
+    <col min="2" max="2" width="8.42578125" customWidth="1"/>
+    <col min="3" max="3" width="35.140625" customWidth="1"/>
+    <col min="4" max="4" width="8.42578125" customWidth="1"/>
+    <col min="5" max="5" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.140625" customWidth="1"/>
+    <col min="7" max="7" width="12" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.42578125" customWidth="1"/>
+    <col min="9" max="9" width="7.140625" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="15.6">
-      <c r="A1" s="37" t="s">
+    <row r="1" spans="1:12" ht="15.75">
+      <c r="A1" s="73" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="37"/>
-      <c r="H1" s="37"/>
-      <c r="I1" s="37"/>
-      <c r="J1" s="37"/>
-      <c r="K1" s="37"/>
-      <c r="L1" s="37"/>
-    </row>
-    <row r="2" spans="1:12" ht="20.399999999999999">
-      <c r="A2" s="38" t="s">
+      <c r="B1" s="73"/>
+      <c r="C1" s="73"/>
+      <c r="D1" s="73"/>
+      <c r="E1" s="73"/>
+      <c r="F1" s="73"/>
+      <c r="G1" s="73"/>
+      <c r="H1" s="73"/>
+      <c r="I1" s="73"/>
+      <c r="J1" s="73"/>
+      <c r="K1" s="73"/>
+      <c r="L1" s="73"/>
+    </row>
+    <row r="2" spans="1:12" ht="20.25">
+      <c r="A2" s="74" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="38"/>
-      <c r="C2" s="38"/>
-      <c r="D2" s="38"/>
-      <c r="E2" s="38"/>
-      <c r="F2" s="38"/>
-      <c r="G2" s="38"/>
-      <c r="H2" s="38"/>
-      <c r="I2" s="38"/>
-      <c r="J2" s="38"/>
-      <c r="K2" s="38"/>
-      <c r="L2" s="38"/>
-    </row>
-    <row r="3" spans="1:12" ht="15.6">
-      <c r="A3" s="37" t="s">
+      <c r="B2" s="74"/>
+      <c r="C2" s="74"/>
+      <c r="D2" s="74"/>
+      <c r="E2" s="74"/>
+      <c r="F2" s="74"/>
+      <c r="G2" s="74"/>
+      <c r="H2" s="74"/>
+      <c r="I2" s="74"/>
+      <c r="J2" s="74"/>
+      <c r="K2" s="74"/>
+      <c r="L2" s="74"/>
+    </row>
+    <row r="3" spans="1:12" ht="15.75">
+      <c r="A3" s="73" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="37"/>
-      <c r="C3" s="37"/>
-      <c r="D3" s="37"/>
-      <c r="E3" s="37"/>
-      <c r="F3" s="37"/>
-      <c r="G3" s="37"/>
-      <c r="H3" s="37"/>
-      <c r="I3" s="37"/>
-      <c r="J3" s="37"/>
-      <c r="K3" s="37"/>
-      <c r="L3" s="37"/>
-    </row>
-    <row r="4" spans="1:12" ht="16.8">
-      <c r="A4" s="39" t="s">
+      <c r="B3" s="73"/>
+      <c r="C3" s="73"/>
+      <c r="D3" s="73"/>
+      <c r="E3" s="73"/>
+      <c r="F3" s="73"/>
+      <c r="G3" s="73"/>
+      <c r="H3" s="73"/>
+      <c r="I3" s="73"/>
+      <c r="J3" s="73"/>
+      <c r="K3" s="73"/>
+      <c r="L3" s="73"/>
+    </row>
+    <row r="4" spans="1:12" ht="15.75">
+      <c r="A4" s="83" t="s">
+        <v>83</v>
+      </c>
+      <c r="B4" s="83"/>
+      <c r="C4" s="83"/>
+      <c r="D4" s="83"/>
+      <c r="E4" s="83"/>
+      <c r="F4" s="83"/>
+      <c r="G4" s="83"/>
+      <c r="H4" s="83"/>
+      <c r="I4" s="83"/>
+      <c r="J4" s="83"/>
+      <c r="K4" s="83"/>
+      <c r="L4" s="83"/>
+    </row>
+    <row r="5" spans="1:12" ht="16.5">
+      <c r="A5" s="65"/>
+      <c r="B5" s="65"/>
+      <c r="C5" s="65"/>
+      <c r="D5" s="65"/>
+      <c r="E5" s="65"/>
+      <c r="F5" s="65"/>
+      <c r="G5" s="65"/>
+      <c r="H5" s="65"/>
+      <c r="I5" s="65"/>
+      <c r="J5" s="65"/>
+      <c r="K5" s="65"/>
+      <c r="L5" s="65"/>
+    </row>
+    <row r="6" spans="1:12" ht="19.5">
+      <c r="A6" s="1"/>
+      <c r="B6" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="39"/>
-      <c r="C4" s="39"/>
-      <c r="D4" s="39"/>
-      <c r="E4" s="39"/>
-      <c r="F4" s="39"/>
-      <c r="G4" s="39"/>
-      <c r="H4" s="39"/>
-      <c r="I4" s="39"/>
-      <c r="J4" s="39"/>
-      <c r="K4" s="39"/>
-      <c r="L4" s="39"/>
-    </row>
-    <row r="5" spans="1:12" ht="19.8">
-      <c r="A5" s="3"/>
-      <c r="B5" s="4" t="s">
+      <c r="C6" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
+      <c r="G6" s="4"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="4"/>
+      <c r="J6" s="5"/>
+      <c r="K6" s="4"/>
+      <c r="L6" s="84" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="16.5">
+      <c r="A7" s="4"/>
+      <c r="B7" s="75" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
-      <c r="H5" s="3"/>
-      <c r="I5" s="6"/>
-      <c r="J5" s="7"/>
-      <c r="K5" s="6"/>
-      <c r="L5" s="8" t="s">
+      <c r="C7" s="75"/>
+      <c r="D7" s="75"/>
+      <c r="E7" s="75"/>
+      <c r="F7" s="75"/>
+      <c r="G7" s="75"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="4"/>
+      <c r="J7" s="4"/>
+      <c r="K7" s="4"/>
+      <c r="L7" s="85" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="15.75">
+      <c r="A8" s="7"/>
+      <c r="B8" s="39" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="6" spans="1:12" ht="17.399999999999999" thickBot="1">
-      <c r="A6" s="6"/>
-      <c r="B6" s="40" t="s">
+      <c r="C8" s="40" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="40"/>
-      <c r="D6" s="40"/>
-      <c r="E6" s="40"/>
-      <c r="F6" s="40"/>
-      <c r="G6" s="40"/>
-      <c r="H6" s="9"/>
-      <c r="I6" s="6"/>
-      <c r="J6" s="6"/>
-      <c r="K6" s="6"/>
-      <c r="L6" s="10" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" ht="16.2" thickBot="1">
-      <c r="A7" s="11"/>
-      <c r="B7" s="12" t="s">
+      <c r="D8" s="41" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="13" t="s">
+      <c r="E8" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="14" t="s">
+      <c r="F8" s="42" t="s">
         <v>15</v>
       </c>
-      <c r="E7" s="15" t="s">
+      <c r="G8" s="42" t="s">
         <v>16</v>
       </c>
-      <c r="F7" s="15" t="s">
+      <c r="H8" s="42" t="s">
+        <v>1</v>
+      </c>
+      <c r="I8" s="43" t="s">
+        <v>2</v>
+      </c>
+      <c r="J8" s="42" t="s">
         <v>17</v>
       </c>
-      <c r="G7" s="15" t="s">
+      <c r="K8" s="42" t="s">
         <v>18</v>
       </c>
-      <c r="H7" s="15" t="s">
+      <c r="L8" s="44" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="36">
+      <c r="B9" s="45">
         <v>1</v>
       </c>
-      <c r="I7" s="16" t="s">
-        <v>2</v>
-      </c>
-      <c r="J7" s="15" t="s">
+      <c r="C9" s="46" t="s">
         <v>19</v>
       </c>
-      <c r="K7" s="15" t="s">
-        <v>20</v>
-      </c>
-      <c r="L7" s="17" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" ht="34.799999999999997">
-      <c r="B8" s="22">
-        <v>1</v>
-      </c>
-      <c r="C8" s="36" t="s">
-        <v>21</v>
-      </c>
-      <c r="D8" s="23">
+      <c r="D9" s="47">
         <f>ROUNDUP(400/3,0)+1</f>
         <v>135</v>
       </c>
-      <c r="E8" s="23">
+      <c r="E9" s="47">
         <v>0.45</v>
       </c>
-      <c r="F8" s="23">
+      <c r="F9" s="47">
         <v>0.45</v>
       </c>
-      <c r="G8" s="23">
+      <c r="G9" s="47">
         <v>0.6</v>
       </c>
-      <c r="H8" s="23">
-        <f>D8*E8*F8*G8</f>
+      <c r="H9" s="47">
+        <f>D9*E9*F9*G9</f>
         <v>16.4025</v>
       </c>
-      <c r="I8" s="24" t="s">
+      <c r="I9" s="48" t="s">
         <v>6</v>
       </c>
-      <c r="J8" s="23">
+      <c r="J9" s="47">
         <v>674.12</v>
       </c>
-      <c r="K8" s="23">
-        <f>H8*J8</f>
+      <c r="K9" s="47">
+        <f>H9*J9</f>
         <v>11057.2533</v>
       </c>
-      <c r="L8" s="25"/>
-    </row>
-    <row r="9" spans="1:12" ht="15.6">
-      <c r="B9" s="20"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
-      <c r="J9" s="2"/>
-      <c r="K9" s="2"/>
-      <c r="L9" s="2"/>
-    </row>
-    <row r="10" spans="1:12" ht="34.799999999999997">
-      <c r="B10" s="20">
+      <c r="L9" s="49"/>
+    </row>
+    <row r="10" spans="1:12" ht="15.75">
+      <c r="B10" s="45"/>
+      <c r="C10" s="49"/>
+      <c r="D10" s="49"/>
+      <c r="E10" s="49"/>
+      <c r="F10" s="49"/>
+      <c r="G10" s="49"/>
+      <c r="H10" s="49"/>
+      <c r="I10" s="49"/>
+      <c r="J10" s="49"/>
+      <c r="K10" s="49"/>
+      <c r="L10" s="49"/>
+    </row>
+    <row r="11" spans="1:12" ht="36">
+      <c r="B11" s="45">
         <v>2</v>
       </c>
-      <c r="C10" s="18" t="s">
+      <c r="C11" s="50" t="s">
+        <v>20</v>
+      </c>
+      <c r="D11" s="51">
+        <f>D9</f>
+        <v>135</v>
+      </c>
+      <c r="E11" s="51">
+        <v>0.3</v>
+      </c>
+      <c r="F11" s="51">
+        <v>0.3</v>
+      </c>
+      <c r="G11" s="51">
+        <v>0.45</v>
+      </c>
+      <c r="H11" s="51">
+        <f>D11*E11*F11*G11</f>
+        <v>5.4675000000000002</v>
+      </c>
+      <c r="I11" s="51" t="s">
+        <v>6</v>
+      </c>
+      <c r="J11" s="51">
+        <v>13351.1</v>
+      </c>
+      <c r="K11" s="51">
+        <f>J11*H11</f>
+        <v>72997.139250000007</v>
+      </c>
+      <c r="L11" s="49"/>
+    </row>
+    <row r="12" spans="1:12" ht="15.75">
+      <c r="B12" s="45"/>
+      <c r="C12" s="52" t="s">
         <v>22</v>
       </c>
-      <c r="D10" s="19">
-        <f>D8</f>
+      <c r="D12" s="51"/>
+      <c r="E12" s="51"/>
+      <c r="F12" s="51"/>
+      <c r="G12" s="51"/>
+      <c r="H12" s="51"/>
+      <c r="I12" s="51"/>
+      <c r="J12" s="51"/>
+      <c r="K12" s="51">
+        <f>0.13*H11*4169.92</f>
+        <v>2963.8748880000003</v>
+      </c>
+      <c r="L12" s="49"/>
+    </row>
+    <row r="13" spans="1:12" ht="15.75">
+      <c r="B13" s="45"/>
+      <c r="C13" s="52" t="s">
+        <v>23</v>
+      </c>
+      <c r="D13" s="51"/>
+      <c r="E13" s="51"/>
+      <c r="F13" s="51"/>
+      <c r="G13" s="51"/>
+      <c r="H13" s="51"/>
+      <c r="I13" s="51"/>
+      <c r="J13" s="53"/>
+      <c r="K13" s="51">
+        <f>0.13*H11*1414.16</f>
+        <v>1005.1495740000001</v>
+      </c>
+      <c r="L13" s="49"/>
+    </row>
+    <row r="14" spans="1:12" ht="15.75">
+      <c r="B14" s="45"/>
+      <c r="C14" s="52" t="s">
+        <v>24</v>
+      </c>
+      <c r="D14" s="51"/>
+      <c r="E14" s="51"/>
+      <c r="F14" s="51"/>
+      <c r="G14" s="51"/>
+      <c r="H14" s="51"/>
+      <c r="I14" s="51"/>
+      <c r="J14" s="53"/>
+      <c r="K14" s="51">
+        <f>0.13*H11*(1652.5+737.97+349.56)</f>
+        <v>1947.5448232500003</v>
+      </c>
+      <c r="L14" s="49"/>
+    </row>
+    <row r="15" spans="1:12" ht="15.75">
+      <c r="B15" s="45"/>
+      <c r="C15" s="52"/>
+      <c r="D15" s="51"/>
+      <c r="E15" s="51"/>
+      <c r="F15" s="51"/>
+      <c r="G15" s="51"/>
+      <c r="H15" s="51"/>
+      <c r="I15" s="51"/>
+      <c r="J15" s="53"/>
+      <c r="K15" s="51"/>
+      <c r="L15" s="49"/>
+    </row>
+    <row r="16" spans="1:12" ht="21.6" customHeight="1">
+      <c r="B16" s="45">
+        <v>3</v>
+      </c>
+      <c r="C16" s="46" t="s">
+        <v>33</v>
+      </c>
+      <c r="D16" s="47">
+        <v>1</v>
+      </c>
+      <c r="E16" s="47">
+        <v>400</v>
+      </c>
+      <c r="F16" s="47"/>
+      <c r="G16" s="47"/>
+      <c r="H16" s="47">
+        <f>PRODUCT(D16:G16)</f>
+        <v>400</v>
+      </c>
+      <c r="I16" s="48" t="s">
+        <v>34</v>
+      </c>
+      <c r="J16" s="47">
+        <v>83.62</v>
+      </c>
+      <c r="K16" s="47">
+        <f>J16*H16</f>
+        <v>33448</v>
+      </c>
+      <c r="L16" s="49"/>
+    </row>
+    <row r="17" spans="1:15" ht="15.75">
+      <c r="B17" s="45"/>
+      <c r="C17" s="52" t="s">
+        <v>35</v>
+      </c>
+      <c r="D17" s="51"/>
+      <c r="E17" s="51"/>
+      <c r="F17" s="51"/>
+      <c r="G17" s="51"/>
+      <c r="H17" s="51"/>
+      <c r="I17" s="51"/>
+      <c r="J17" s="51"/>
+      <c r="K17" s="51">
+        <f>0.13*H16*1992.14/100</f>
+        <v>1035.9128000000001</v>
+      </c>
+      <c r="L17" s="49"/>
+    </row>
+    <row r="18" spans="1:15" ht="15.75">
+      <c r="B18" s="45"/>
+      <c r="C18" s="52"/>
+      <c r="D18" s="51"/>
+      <c r="E18" s="51"/>
+      <c r="F18" s="51"/>
+      <c r="G18" s="51"/>
+      <c r="H18" s="51"/>
+      <c r="I18" s="51"/>
+      <c r="J18" s="53"/>
+      <c r="K18" s="51"/>
+      <c r="L18" s="49"/>
+    </row>
+    <row r="19" spans="1:15" ht="36">
+      <c r="B19" s="45">
+        <v>4</v>
+      </c>
+      <c r="C19" s="54" t="s">
+        <v>27</v>
+      </c>
+      <c r="D19" s="51"/>
+      <c r="E19" s="55" t="s">
+        <v>78</v>
+      </c>
+      <c r="F19" s="56"/>
+      <c r="G19" s="55" t="s">
+        <v>77</v>
+      </c>
+      <c r="H19" s="51"/>
+      <c r="I19" s="51"/>
+      <c r="J19" s="51"/>
+      <c r="K19" s="51"/>
+      <c r="L19" s="49"/>
+    </row>
+    <row r="20" spans="1:15" ht="15.75">
+      <c r="B20" s="49"/>
+      <c r="C20" s="61" t="s">
+        <v>82</v>
+      </c>
+      <c r="D20" s="51">
+        <f>D11</f>
         <v>135</v>
       </c>
-      <c r="E10" s="19">
-        <v>0.3</v>
-      </c>
-      <c r="F10" s="19">
-        <v>0.3</v>
-      </c>
-      <c r="G10" s="19">
-        <v>0.45</v>
-      </c>
-      <c r="H10" s="19">
-        <f>D10*E10*F10*G10</f>
-        <v>5.4675000000000002</v>
-      </c>
-      <c r="I10" s="19" t="s">
-        <v>6</v>
-      </c>
-      <c r="J10" s="19">
-        <v>13351.1</v>
-      </c>
-      <c r="K10" s="19">
-        <f>J10*H10</f>
-        <v>72997.139250000007</v>
-      </c>
-      <c r="L10" s="2"/>
-    </row>
-    <row r="11" spans="1:12" ht="15.6">
-      <c r="B11" s="20"/>
-      <c r="C11" s="21" t="s">
-        <v>24</v>
-      </c>
-      <c r="D11" s="19"/>
-      <c r="E11" s="19"/>
-      <c r="F11" s="19"/>
-      <c r="G11" s="19"/>
-      <c r="H11" s="19"/>
-      <c r="I11" s="19"/>
-      <c r="J11" s="19"/>
-      <c r="K11" s="19">
-        <f>0.13*H10*4169.92</f>
-        <v>2963.8748880000003</v>
-      </c>
-      <c r="L11" s="2"/>
-    </row>
-    <row r="12" spans="1:12" ht="15.6">
-      <c r="B12" s="20"/>
-      <c r="C12" s="21" t="s">
-        <v>25</v>
-      </c>
-      <c r="D12" s="19"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="19"/>
-      <c r="G12" s="19"/>
-      <c r="H12" s="19"/>
-      <c r="I12" s="19"/>
-      <c r="J12" s="1"/>
-      <c r="K12" s="19">
-        <f>0.13*H10*1414.16</f>
-        <v>1005.1495740000001</v>
-      </c>
-      <c r="L12" s="2"/>
-    </row>
-    <row r="13" spans="1:12" ht="15.6">
-      <c r="B13" s="20"/>
-      <c r="C13" s="21" t="s">
-        <v>26</v>
-      </c>
-      <c r="D13" s="19"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="19"/>
-      <c r="G13" s="19"/>
-      <c r="H13" s="19"/>
-      <c r="I13" s="19"/>
-      <c r="J13" s="1"/>
-      <c r="K13" s="19">
-        <f>0.13*H10*(1652.5+737.97+349.56)</f>
-        <v>1947.5448232500003</v>
-      </c>
-      <c r="L13" s="2"/>
-    </row>
-    <row r="14" spans="1:12" ht="16.2" thickBot="1">
-      <c r="B14" s="20"/>
-      <c r="C14" s="21"/>
-      <c r="D14" s="19"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="19"/>
-      <c r="G14" s="19"/>
-      <c r="H14" s="19"/>
-      <c r="I14" s="19"/>
-      <c r="J14" s="1"/>
-      <c r="K14" s="19"/>
-      <c r="L14" s="2"/>
-    </row>
-    <row r="15" spans="1:12" ht="21.6" customHeight="1">
-      <c r="B15" s="22">
-        <v>3</v>
-      </c>
-      <c r="C15" s="36" t="s">
-        <v>40</v>
-      </c>
-      <c r="D15" s="23">
-        <v>1</v>
-      </c>
-      <c r="E15" s="23">
-        <v>400</v>
-      </c>
-      <c r="F15" s="23"/>
-      <c r="G15" s="23"/>
-      <c r="H15" s="23">
-        <f>PRODUCT(D15:G15)</f>
-        <v>400</v>
-      </c>
-      <c r="I15" s="24" t="s">
-        <v>41</v>
-      </c>
-      <c r="J15" s="23">
-        <v>83.62</v>
-      </c>
-      <c r="K15" s="23">
-        <f>J15*H15</f>
-        <v>33448</v>
-      </c>
-      <c r="L15" s="25"/>
-    </row>
-    <row r="16" spans="1:12" ht="15.6">
-      <c r="B16" s="20"/>
-      <c r="C16" s="21" t="s">
-        <v>42</v>
-      </c>
-      <c r="D16" s="19"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="19"/>
-      <c r="G16" s="19"/>
-      <c r="H16" s="19"/>
-      <c r="I16" s="19"/>
-      <c r="J16" s="19"/>
-      <c r="K16" s="19">
-        <f>0.13*H15*1992.14/100</f>
-        <v>1035.9128000000001</v>
-      </c>
-      <c r="L16" s="2"/>
-    </row>
-    <row r="17" spans="2:15" ht="15.6">
-      <c r="B17" s="20"/>
-      <c r="C17" s="21"/>
-      <c r="D17" s="19"/>
-      <c r="E17" s="19"/>
-      <c r="F17" s="19"/>
-      <c r="G17" s="19"/>
-      <c r="H17" s="19"/>
-      <c r="I17" s="19"/>
-      <c r="J17" s="1"/>
-      <c r="K17" s="19"/>
-      <c r="L17" s="2"/>
-    </row>
-    <row r="18" spans="2:15" ht="34.799999999999997">
-      <c r="B18" s="20">
-        <v>4</v>
-      </c>
-      <c r="C18" s="32" t="s">
-        <v>29</v>
-      </c>
-      <c r="D18" s="19"/>
-      <c r="E18" s="19"/>
-      <c r="F18" s="19"/>
-      <c r="G18" s="19" t="s">
-        <v>34</v>
-      </c>
-      <c r="H18" s="19"/>
-      <c r="I18" s="19"/>
-      <c r="J18" s="19"/>
-      <c r="K18" s="19"/>
-      <c r="L18" s="2"/>
-    </row>
-    <row r="19" spans="2:15" ht="15.6">
-      <c r="B19" s="29"/>
-      <c r="C19" s="30" t="s">
-        <v>45</v>
-      </c>
-      <c r="D19" s="19">
-        <f>D10</f>
-        <v>135</v>
-      </c>
-      <c r="E19" s="19">
+      <c r="E20" s="51">
         <f>6.5/3.28</f>
         <v>1.9817073170731709</v>
       </c>
-      <c r="F19" s="19"/>
-      <c r="G19" s="19">
+      <c r="F20" s="51"/>
+      <c r="G20" s="51">
         <v>1.19</v>
       </c>
-      <c r="H19" s="19">
-        <f>D19*E19*G19</f>
+      <c r="H20" s="51">
+        <f>D20*E20*G20</f>
         <v>318.36128048780489</v>
       </c>
-      <c r="I19" s="19" t="s">
-        <v>28</v>
-      </c>
-      <c r="J19" s="19">
+      <c r="I20" s="51" t="s">
+        <v>26</v>
+      </c>
+      <c r="J20" s="51">
         <v>93</v>
       </c>
-      <c r="K19" s="19">
-        <f>H19*J19</f>
+      <c r="K20" s="51">
+        <f>H20*J20</f>
         <v>29607.599085365855</v>
       </c>
-      <c r="L19" s="29"/>
-    </row>
-    <row r="20" spans="2:15" ht="15.6">
-      <c r="B20" s="29"/>
-      <c r="C20" s="30" t="s">
-        <v>23</v>
-      </c>
-      <c r="D20" s="19"/>
-      <c r="E20" s="19"/>
-      <c r="F20" s="19"/>
-      <c r="G20" s="19"/>
-      <c r="H20" s="19"/>
-      <c r="I20" s="19"/>
-      <c r="J20" s="19"/>
-      <c r="K20" s="19">
-        <f>0.13*K19</f>
+      <c r="L20" s="49"/>
+    </row>
+    <row r="21" spans="1:15" ht="15.75">
+      <c r="B21" s="49"/>
+      <c r="C21" s="52" t="s">
+        <v>21</v>
+      </c>
+      <c r="D21" s="51"/>
+      <c r="E21" s="51"/>
+      <c r="F21" s="51"/>
+      <c r="G21" s="51"/>
+      <c r="H21" s="51"/>
+      <c r="I21" s="51"/>
+      <c r="J21" s="51"/>
+      <c r="K21" s="51">
+        <f>0.13*K20</f>
         <v>3848.9878810975611</v>
       </c>
-      <c r="L20" s="29"/>
-    </row>
-    <row r="21" spans="2:15" ht="15.6">
-      <c r="B21" s="29"/>
-      <c r="C21" s="33"/>
-      <c r="D21" s="19"/>
-      <c r="E21" s="19"/>
-      <c r="F21" s="19"/>
-      <c r="G21" s="19"/>
-      <c r="H21" s="19"/>
-      <c r="I21" s="19"/>
-      <c r="J21" s="19"/>
-      <c r="K21" s="19"/>
-      <c r="L21" s="29"/>
-    </row>
-    <row r="22" spans="2:15" ht="31.2">
-      <c r="B22" s="29"/>
-      <c r="C22" s="35" t="s">
-        <v>33</v>
-      </c>
-      <c r="D22" s="19">
+      <c r="L21" s="49"/>
+    </row>
+    <row r="22" spans="1:15" ht="31.5">
+      <c r="B22" s="49"/>
+      <c r="C22" s="60" t="s">
+        <v>79</v>
+      </c>
+      <c r="D22" s="51">
         <v>1</v>
       </c>
-      <c r="E22" s="19">
+      <c r="E22" s="51">
         <v>400</v>
       </c>
-      <c r="F22" s="19"/>
-      <c r="G22" s="19">
+      <c r="F22" s="51"/>
+      <c r="G22" s="51">
         <f>4.5/3.281</f>
         <v>1.3715330691862238</v>
       </c>
-      <c r="H22" s="19">
+      <c r="H22" s="51">
         <f>E22*G22</f>
         <v>548.61322767448951</v>
       </c>
-      <c r="I22" s="19" t="s">
+      <c r="I22" s="51" t="s">
         <v>5</v>
       </c>
-      <c r="J22" s="19">
+      <c r="J22" s="51">
         <v>501</v>
       </c>
-      <c r="K22" s="19">
+      <c r="K22" s="51">
         <f>H22*J22</f>
         <v>274855.22706491925</v>
       </c>
-      <c r="L22" s="29"/>
-    </row>
-    <row r="23" spans="2:15" ht="15.6">
-      <c r="B23" s="29"/>
-      <c r="C23" s="30" t="s">
-        <v>23</v>
-      </c>
-      <c r="D23" s="29"/>
-      <c r="E23" s="29"/>
-      <c r="F23" s="29"/>
-      <c r="G23" s="29"/>
-      <c r="H23" s="29"/>
-      <c r="I23" s="29"/>
-      <c r="J23" s="29"/>
-      <c r="K23" s="31">
+      <c r="L22" s="49"/>
+    </row>
+    <row r="23" spans="1:15" ht="15.75">
+      <c r="B23" s="49"/>
+      <c r="C23" s="52" t="s">
+        <v>21</v>
+      </c>
+      <c r="D23" s="49"/>
+      <c r="E23" s="49"/>
+      <c r="F23" s="49"/>
+      <c r="G23" s="49"/>
+      <c r="H23" s="49"/>
+      <c r="I23" s="49"/>
+      <c r="J23" s="49"/>
+      <c r="K23" s="51">
         <f>0.13*K22</f>
         <v>35731.179518439501</v>
       </c>
-      <c r="L23" s="29"/>
-    </row>
-    <row r="24" spans="2:15" ht="15.6">
-      <c r="B24" s="29"/>
-      <c r="C24" s="30"/>
-      <c r="D24" s="29"/>
-      <c r="E24" s="29"/>
-      <c r="F24" s="29"/>
-      <c r="G24" s="29"/>
-      <c r="H24" s="29"/>
-      <c r="I24" s="29"/>
-      <c r="J24" s="29"/>
-      <c r="K24" s="31"/>
-      <c r="L24" s="29"/>
+      <c r="L23" s="49"/>
+    </row>
+    <row r="24" spans="1:15" ht="15.75">
+      <c r="B24" s="49"/>
+      <c r="C24" s="52"/>
+      <c r="D24" s="49"/>
+      <c r="E24" s="49"/>
+      <c r="F24" s="49"/>
+      <c r="G24" s="49"/>
+      <c r="H24" s="49"/>
+      <c r="I24" s="49"/>
+      <c r="J24" s="49"/>
+      <c r="K24" s="51"/>
+      <c r="L24" s="49"/>
       <c r="O24" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="25" spans="2:15" ht="15.6">
-      <c r="B25" s="29"/>
-      <c r="C25" s="30" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" ht="15.75">
+      <c r="B25" s="49"/>
+      <c r="C25" s="61" t="s">
+        <v>80</v>
+      </c>
+      <c r="D25" s="57">
+        <v>5</v>
+      </c>
+      <c r="E25" s="49"/>
+      <c r="F25" s="49"/>
+      <c r="G25" s="49"/>
+      <c r="H25" s="51">
+        <f>D25</f>
+        <v>5</v>
+      </c>
+      <c r="I25" s="51" t="s">
+        <v>28</v>
+      </c>
+      <c r="J25" s="51">
+        <v>1035</v>
+      </c>
+      <c r="K25" s="51">
+        <f>H25*J25</f>
+        <v>5175</v>
+      </c>
+      <c r="L25" s="49"/>
+      <c r="O25" s="8" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" ht="15.75">
+      <c r="B26" s="49"/>
+      <c r="C26" s="61" t="s">
+        <v>81</v>
+      </c>
+      <c r="D26" s="57">
+        <v>15</v>
+      </c>
+      <c r="E26" s="49"/>
+      <c r="F26" s="49"/>
+      <c r="G26" s="49"/>
+      <c r="H26" s="51">
+        <f>D26</f>
+        <v>15</v>
+      </c>
+      <c r="I26" s="51" t="s">
+        <v>28</v>
+      </c>
+      <c r="J26" s="51">
+        <v>825</v>
+      </c>
+      <c r="K26" s="51">
+        <f>H26*J26</f>
+        <v>12375</v>
+      </c>
+      <c r="L26" s="49"/>
+      <c r="O26" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="D25" s="34">
-        <v>12</v>
-      </c>
-      <c r="E25" s="29"/>
-      <c r="F25" s="29"/>
-      <c r="G25" s="29"/>
-      <c r="H25" s="19">
-        <f>D25</f>
-        <v>12</v>
-      </c>
-      <c r="I25" s="19" t="s">
-        <v>30</v>
-      </c>
-      <c r="J25" s="19">
-        <v>1020</v>
-      </c>
-      <c r="K25" s="31">
-        <f>H25*J25</f>
-        <v>12240</v>
-      </c>
-      <c r="L25" s="29"/>
-      <c r="O25" s="29" t="s">
+    </row>
+    <row r="27" spans="1:15" ht="15.75">
+      <c r="B27" s="49"/>
+      <c r="C27" s="52"/>
+      <c r="D27" s="57"/>
+      <c r="E27" s="49"/>
+      <c r="F27" s="49"/>
+      <c r="G27" s="49"/>
+      <c r="H27" s="51"/>
+      <c r="I27" s="51"/>
+      <c r="J27" s="51"/>
+      <c r="K27" s="51"/>
+      <c r="L27" s="49"/>
+      <c r="O27" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" ht="15.75">
+      <c r="B28" s="45">
+        <v>5</v>
+      </c>
+      <c r="C28" s="52" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="26" spans="2:15" ht="15.6">
-      <c r="B26" s="29"/>
-      <c r="C26" s="30" t="s">
-        <v>32</v>
-      </c>
-      <c r="D26" s="34">
-        <v>19</v>
-      </c>
-      <c r="E26" s="29"/>
-      <c r="F26" s="29"/>
-      <c r="G26" s="29"/>
-      <c r="H26" s="19">
-        <f>D26</f>
-        <v>19</v>
-      </c>
-      <c r="I26" s="19" t="s">
-        <v>30</v>
-      </c>
-      <c r="J26" s="19">
-        <v>810</v>
-      </c>
-      <c r="K26" s="31">
-        <f>H26*J26</f>
-        <v>15390</v>
-      </c>
-      <c r="L26" s="29"/>
-      <c r="O26" s="29" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="27" spans="2:15" ht="16.2" thickBot="1">
-      <c r="B27" s="29"/>
-      <c r="C27" s="30"/>
-      <c r="D27" s="34"/>
-      <c r="E27" s="29"/>
-      <c r="F27" s="29"/>
-      <c r="G27" s="29"/>
-      <c r="H27" s="31"/>
-      <c r="I27" s="31"/>
-      <c r="J27" s="31"/>
-      <c r="K27" s="31"/>
-      <c r="L27" s="29"/>
-      <c r="O27" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="28" spans="2:15" ht="15.6">
-      <c r="B28" s="20">
-        <v>5</v>
-      </c>
-      <c r="C28" s="30" t="s">
-        <v>43</v>
-      </c>
-      <c r="D28" s="34">
+      <c r="D28" s="57">
         <v>1</v>
       </c>
-      <c r="E28" s="29"/>
-      <c r="F28" s="29"/>
-      <c r="G28" s="29"/>
-      <c r="H28" s="23">
+      <c r="E28" s="49"/>
+      <c r="F28" s="49"/>
+      <c r="G28" s="49"/>
+      <c r="H28" s="47">
         <f>PRODUCT(D28:G28)</f>
         <v>1</v>
       </c>
-      <c r="I28" s="31" t="s">
-        <v>44</v>
-      </c>
-      <c r="J28" s="31">
+      <c r="I28" s="51" t="s">
+        <v>37</v>
+      </c>
+      <c r="J28" s="51">
         <v>500</v>
       </c>
-      <c r="K28" s="19">
+      <c r="K28" s="51">
         <f>H28*J28</f>
         <v>500</v>
       </c>
-      <c r="L28" s="29"/>
-    </row>
-    <row r="29" spans="2:15" ht="15.6">
-      <c r="B29" s="29"/>
-      <c r="C29" s="30"/>
-      <c r="D29" s="34"/>
-      <c r="E29" s="29"/>
-      <c r="F29" s="29"/>
-      <c r="G29" s="29"/>
-      <c r="H29" s="31"/>
-      <c r="I29" s="31"/>
-      <c r="J29" s="31"/>
-      <c r="K29" s="31"/>
-      <c r="L29" s="29"/>
-    </row>
-    <row r="30" spans="2:15" ht="17.399999999999999">
-      <c r="B30" s="26"/>
-      <c r="C30" s="27" t="s">
+      <c r="L28" s="49"/>
+    </row>
+    <row r="29" spans="1:15" ht="15.75">
+      <c r="B29" s="49"/>
+      <c r="C29" s="52"/>
+      <c r="D29" s="57"/>
+      <c r="E29" s="49"/>
+      <c r="F29" s="49"/>
+      <c r="G29" s="49"/>
+      <c r="H29" s="51"/>
+      <c r="I29" s="51"/>
+      <c r="J29" s="51"/>
+      <c r="K29" s="51"/>
+      <c r="L29" s="49"/>
+    </row>
+    <row r="30" spans="1:15" ht="18.75">
+      <c r="B30" s="49"/>
+      <c r="C30" s="58" t="s">
         <v>4</v>
       </c>
-      <c r="D30" s="26"/>
-      <c r="E30" s="26"/>
-      <c r="F30" s="26"/>
-      <c r="G30" s="26"/>
-      <c r="H30" s="26"/>
-      <c r="I30" s="26"/>
-      <c r="J30" s="26"/>
-      <c r="K30" s="28">
-        <f>SUM(K8:K28)</f>
-        <v>496627.86818507221</v>
-      </c>
-      <c r="L30" s="26"/>
-    </row>
-    <row r="33" spans="3:9">
-      <c r="G33">
+      <c r="D30" s="49"/>
+      <c r="E30" s="49"/>
+      <c r="F30" s="49"/>
+      <c r="G30" s="49"/>
+      <c r="H30" s="49"/>
+      <c r="I30" s="49"/>
+      <c r="J30" s="49"/>
+      <c r="K30" s="59">
+        <f>SUM(K9:K28)</f>
+        <v>486547.86818507221</v>
+      </c>
+      <c r="L30" s="49"/>
+    </row>
+    <row r="32" spans="1:15" s="38" customFormat="1">
+      <c r="A32" s="31"/>
+      <c r="C32" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="D32" s="66">
+        <f>K30</f>
+        <v>486547.86818507221</v>
+      </c>
+      <c r="E32" s="66"/>
+      <c r="F32" s="64"/>
+      <c r="G32" s="34"/>
+      <c r="H32" s="31"/>
+      <c r="I32" s="35"/>
+      <c r="J32" s="36"/>
+      <c r="K32" s="37"/>
+    </row>
+    <row r="33" spans="3:9" hidden="1">
+      <c r="C33" s="62" t="s">
+        <v>72</v>
+      </c>
+      <c r="D33" s="67">
+        <v>480000</v>
+      </c>
+      <c r="E33" s="68"/>
+      <c r="F33" s="63"/>
+    </row>
+    <row r="34" spans="3:9" hidden="1">
+      <c r="C34" s="32" t="s">
+        <v>73</v>
+      </c>
+      <c r="D34" s="69">
+        <f>D33-D36-D37</f>
+        <v>456000</v>
+      </c>
+      <c r="E34" s="70"/>
+      <c r="F34" s="33">
+        <f>D34/D32*100</f>
+        <v>93.721508163416217</v>
+      </c>
+      <c r="G34" s="28"/>
+    </row>
+    <row r="35" spans="3:9" hidden="1">
+      <c r="C35" s="32" t="s">
+        <v>74</v>
+      </c>
+      <c r="D35" s="66">
+        <f>D32-D34</f>
+        <v>30547.868185072206</v>
+      </c>
+      <c r="E35" s="66"/>
+      <c r="F35" s="33">
+        <f>100-F34</f>
+        <v>6.2784918365837825</v>
+      </c>
+    </row>
+    <row r="36" spans="3:9" hidden="1">
+      <c r="C36" s="32" t="s">
+        <v>75</v>
+      </c>
+      <c r="D36" s="71">
+        <f>D33*0.03</f>
+        <v>14400</v>
+      </c>
+      <c r="E36" s="72"/>
+      <c r="F36" s="33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="3:9" hidden="1">
+      <c r="C37" s="32" t="s">
+        <v>76</v>
+      </c>
+      <c r="D37" s="71">
+        <f>D33*0.02</f>
+        <v>9600</v>
+      </c>
+      <c r="E37" s="72"/>
+      <c r="F37" s="33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="3:9">
+      <c r="G40">
         <f>400/650*20</f>
         <v>12.307692307692308</v>
       </c>
-      <c r="H33">
+      <c r="H40">
         <f>400/650*30</f>
         <v>18.461538461538463</v>
       </c>
     </row>
-    <row r="34" spans="3:9">
-      <c r="F34">
+    <row r="41" spans="3:9">
+      <c r="F41">
         <v>650</v>
       </c>
-      <c r="G34">
+      <c r="G41">
         <v>400</v>
       </c>
-      <c r="H34">
+      <c r="H41">
         <v>650</v>
       </c>
-      <c r="I34">
+      <c r="I41">
         <v>400</v>
       </c>
     </row>
-    <row r="35" spans="3:9">
-      <c r="F35">
+    <row r="42" spans="3:9">
+      <c r="F42">
         <v>20</v>
       </c>
-      <c r="G35">
+      <c r="G42">
         <v>12</v>
       </c>
-      <c r="H35">
+      <c r="H42">
         <v>30</v>
       </c>
-      <c r="I35">
+      <c r="I42">
         <v>19</v>
       </c>
     </row>
-    <row r="37" spans="3:9">
-      <c r="C37" s="69">
+    <row r="44" spans="3:9">
+      <c r="C44" s="30">
         <f>Sheet1!I16/10*H22</f>
         <v>1457247.7141115514</v>
       </c>
-      <c r="F37">
+      <c r="F44">
         <v>10</v>
       </c>
-      <c r="G37">
+      <c r="G44">
         <v>400</v>
       </c>
-      <c r="H37">
+      <c r="H44">
         <v>10</v>
       </c>
-      <c r="I37">
+      <c r="I44">
         <v>400</v>
       </c>
     </row>
-    <row r="38" spans="3:9">
-      <c r="F38">
+    <row r="45" spans="3:9">
+      <c r="F45">
         <v>7</v>
       </c>
-      <c r="G38">
-        <f>G37/F37*F38</f>
+      <c r="G45">
+        <f>G44/F44*F45</f>
         <v>280</v>
       </c>
-      <c r="H38">
+      <c r="H45">
         <v>5</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="11">
+    <mergeCell ref="D37:E37"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:L2"/>
     <mergeCell ref="A3:L3"/>
     <mergeCell ref="A4:L4"/>
-    <mergeCell ref="B6:G6"/>
+    <mergeCell ref="B7:G7"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="D34:E34"/>
+    <mergeCell ref="D35:E35"/>
+    <mergeCell ref="D36:E36"/>
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup scale="80" orientation="landscape" verticalDpi="1200" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="80" orientation="landscape" verticalDpi="1200" r:id="rId1"/>
+  <headerFooter>
+    <oddFooter>&amp;LPrepared By:&amp;CChecked By:&amp;RApproved By:</oddFooter>
+  </headerFooter>
   <colBreaks count="1" manualBreakCount="1">
     <brk id="12" max="1048575" man="1"/>
   </colBreaks>
@@ -2446,316 +2577,316 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="B2:K20"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="4" max="4" width="21.6640625" customWidth="1"/>
-    <col min="7" max="7" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.7109375" customWidth="1"/>
+    <col min="7" max="7" width="9.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:11" ht="15.6">
-      <c r="B2" s="41">
+    <row r="2" spans="2:11">
+      <c r="B2" s="9">
         <v>297</v>
       </c>
-      <c r="C2" s="42" t="s">
+      <c r="C2" s="79" t="s">
+        <v>38</v>
+      </c>
+      <c r="D2" s="80"/>
+      <c r="E2" s="80"/>
+      <c r="F2" s="80"/>
+      <c r="G2" s="80"/>
+      <c r="H2" s="80"/>
+      <c r="I2" s="80"/>
+      <c r="J2" s="29"/>
+      <c r="K2" s="29"/>
+    </row>
+    <row r="3" spans="2:11">
+      <c r="B3" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="C3" s="81" t="s">
+        <v>40</v>
+      </c>
+      <c r="D3" s="80"/>
+      <c r="E3" s="80"/>
+      <c r="F3" s="80"/>
+      <c r="G3" s="80"/>
+      <c r="H3" s="80"/>
+      <c r="I3" s="80"/>
+    </row>
+    <row r="4" spans="2:11">
+      <c r="C4" s="80" t="s">
+        <v>41</v>
+      </c>
+      <c r="D4" s="80"/>
+      <c r="E4" s="80"/>
+      <c r="F4" s="80"/>
+      <c r="G4" s="80"/>
+      <c r="H4" s="80"/>
+      <c r="I4" s="80"/>
+    </row>
+    <row r="5" spans="2:11">
+      <c r="C5" s="80" t="s">
+        <v>42</v>
+      </c>
+      <c r="D5" s="80"/>
+      <c r="E5" s="80"/>
+      <c r="F5" s="80"/>
+      <c r="G5" s="80"/>
+      <c r="H5" s="80"/>
+      <c r="I5" s="80"/>
+    </row>
+    <row r="6" spans="2:11">
+      <c r="C6" s="82" t="s">
+        <v>43</v>
+      </c>
+      <c r="D6" s="82"/>
+      <c r="E6" s="82"/>
+      <c r="F6" s="82"/>
+      <c r="G6" s="82"/>
+      <c r="H6" s="82"/>
+      <c r="I6" s="82"/>
+    </row>
+    <row r="7" spans="2:11" ht="63">
+      <c r="C7" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="E7" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="D2" s="43"/>
-      <c r="E2" s="43"/>
-      <c r="F2" s="43"/>
-      <c r="G2" s="43"/>
-      <c r="H2" s="43"/>
-      <c r="I2" s="43"/>
-      <c r="J2" s="68"/>
-      <c r="K2" s="68"/>
-    </row>
-    <row r="3" spans="2:11" ht="15">
-      <c r="B3" s="44" t="s">
+      <c r="F7" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="C3" s="45" t="s">
+      <c r="G7" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="D3" s="43"/>
-      <c r="E3" s="43"/>
-      <c r="F3" s="43"/>
-      <c r="G3" s="43"/>
-      <c r="H3" s="43"/>
-      <c r="I3" s="43"/>
-    </row>
-    <row r="4" spans="2:11" ht="15">
-      <c r="C4" s="43" t="s">
+      <c r="H7" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="D4" s="43"/>
-      <c r="E4" s="43"/>
-      <c r="F4" s="43"/>
-      <c r="G4" s="43"/>
-      <c r="H4" s="43"/>
-      <c r="I4" s="43"/>
-    </row>
-    <row r="5" spans="2:11" ht="15">
-      <c r="C5" s="43" t="s">
+      <c r="I7" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="D5" s="43"/>
-      <c r="E5" s="43"/>
-      <c r="F5" s="43"/>
-      <c r="G5" s="43"/>
-      <c r="H5" s="43"/>
-      <c r="I5" s="43"/>
-    </row>
-    <row r="6" spans="2:11">
-      <c r="C6" s="46" t="s">
+    </row>
+    <row r="8" spans="2:11" ht="16.5">
+      <c r="C8" s="76" t="s">
         <v>51</v>
       </c>
-      <c r="D6" s="46"/>
-      <c r="E6" s="46"/>
-      <c r="F6" s="46"/>
-      <c r="G6" s="46"/>
-      <c r="H6" s="46"/>
-      <c r="I6" s="46"/>
-    </row>
-    <row r="7" spans="2:11" ht="64.8">
-      <c r="C7" s="48" t="s">
+      <c r="D8" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="D7" s="48" t="s">
+      <c r="E8" s="28">
+        <v>7</v>
+      </c>
+      <c r="F8" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="E7" s="48" t="s">
-        <v>54</v>
-      </c>
-      <c r="F7" s="48" t="s">
-        <v>55</v>
-      </c>
-      <c r="G7" s="48" t="s">
-        <v>56</v>
-      </c>
-      <c r="H7" s="48" t="s">
-        <v>57</v>
-      </c>
-      <c r="I7" s="48" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="8" spans="2:11" ht="16.8">
-      <c r="C8" s="50" t="s">
-        <v>59</v>
-      </c>
-      <c r="D8" s="51" t="s">
-        <v>60</v>
-      </c>
-      <c r="E8" s="67">
-        <v>7</v>
-      </c>
-      <c r="F8" s="52" t="s">
-        <v>61</v>
-      </c>
-      <c r="G8" s="53">
+      <c r="G8" s="16">
         <v>1245</v>
       </c>
-      <c r="H8" s="67">
+      <c r="H8" s="28">
         <f t="shared" ref="H8:H14" si="0">FLOOR(E8*G8,0.01)</f>
         <v>8715</v>
       </c>
-      <c r="I8" s="67"/>
-    </row>
-    <row r="9" spans="2:11" ht="16.8">
-      <c r="C9" s="54"/>
-      <c r="D9" s="55" t="s">
-        <v>62</v>
-      </c>
-      <c r="E9" s="67">
+      <c r="I8" s="28"/>
+    </row>
+    <row r="9" spans="2:11" ht="16.5">
+      <c r="C9" s="78"/>
+      <c r="D9" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="E9" s="28">
         <v>5</v>
       </c>
-      <c r="F9" s="56" t="s">
-        <v>61</v>
-      </c>
-      <c r="G9" s="57">
+      <c r="F9" s="18" t="s">
+        <v>53</v>
+      </c>
+      <c r="G9" s="19">
         <v>935</v>
       </c>
-      <c r="H9" s="67">
+      <c r="H9" s="28">
         <f t="shared" si="0"/>
         <v>4675</v>
       </c>
-      <c r="I9" s="67">
+      <c r="I9" s="28">
         <f>SUM(H8+H9)</f>
         <v>13390</v>
       </c>
     </row>
-    <row r="10" spans="2:11" ht="16.8">
-      <c r="C10" s="50" t="s">
-        <v>63</v>
-      </c>
-      <c r="D10" s="51" t="s">
-        <v>64</v>
-      </c>
-      <c r="E10" s="67">
+    <row r="10" spans="2:11" ht="16.5">
+      <c r="C10" s="76" t="s">
+        <v>55</v>
+      </c>
+      <c r="D10" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="E10" s="28">
         <f>0*35.51</f>
         <v>0</v>
       </c>
-      <c r="F10" s="52" t="s">
-        <v>65</v>
-      </c>
-      <c r="G10" s="53">
+      <c r="F10" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="G10" s="16">
         <v>93</v>
       </c>
-      <c r="H10" s="67">
+      <c r="H10" s="28">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I10" s="67"/>
-    </row>
-    <row r="11" spans="2:11" ht="16.8">
-      <c r="C11" s="58"/>
-      <c r="D11" s="59" t="s">
-        <v>66</v>
-      </c>
-      <c r="E11" s="67">
+      <c r="I10" s="28"/>
+    </row>
+    <row r="11" spans="2:11" ht="16.5">
+      <c r="C11" s="77"/>
+      <c r="D11" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="E11" s="28">
         <v>32.06</v>
       </c>
-      <c r="F11" s="52" t="s">
-        <v>65</v>
-      </c>
-      <c r="G11" s="60">
+      <c r="F11" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="G11" s="21">
         <v>93</v>
       </c>
-      <c r="H11" s="67">
+      <c r="H11" s="28">
         <f>FLOOR(E11*G11,0.01)</f>
         <v>2981.58</v>
       </c>
-      <c r="I11" s="67"/>
-    </row>
-    <row r="12" spans="2:11" ht="16.8">
-      <c r="C12" s="58"/>
-      <c r="D12" s="59" t="s">
-        <v>67</v>
-      </c>
-      <c r="E12" s="67">
+      <c r="I11" s="28"/>
+    </row>
+    <row r="12" spans="2:11" ht="16.5">
+      <c r="C12" s="77"/>
+      <c r="D12" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="E12" s="28">
         <v>25.19</v>
       </c>
-      <c r="F12" s="52" t="s">
-        <v>65</v>
-      </c>
-      <c r="G12" s="60">
+      <c r="F12" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="G12" s="21">
         <v>93</v>
       </c>
-      <c r="H12" s="67">
+      <c r="H12" s="28">
         <f t="shared" si="0"/>
         <v>2342.67</v>
       </c>
-      <c r="I12" s="67"/>
-    </row>
-    <row r="13" spans="2:11" ht="27.6">
-      <c r="C13" s="58"/>
-      <c r="D13" s="61" t="s">
-        <v>68</v>
-      </c>
-      <c r="E13" s="67">
+      <c r="I12" s="28"/>
+    </row>
+    <row r="13" spans="2:11" ht="28.5">
+      <c r="C13" s="77"/>
+      <c r="D13" s="22" t="s">
+        <v>60</v>
+      </c>
+      <c r="E13" s="28">
         <f>0*14.76</f>
         <v>0</v>
       </c>
-      <c r="F13" s="52" t="s">
-        <v>65</v>
-      </c>
-      <c r="G13" s="60">
+      <c r="F13" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="G13" s="21">
         <v>154</v>
       </c>
-      <c r="H13" s="67">
+      <c r="H13" s="28">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I13" s="67"/>
-    </row>
-    <row r="14" spans="2:11" ht="27.6">
-      <c r="C14" s="54"/>
-      <c r="D14" s="61" t="s">
-        <v>69</v>
-      </c>
-      <c r="E14" s="67">
+      <c r="I13" s="28"/>
+    </row>
+    <row r="14" spans="2:11" ht="28.5">
+      <c r="C14" s="78"/>
+      <c r="D14" s="22" t="s">
+        <v>61</v>
+      </c>
+      <c r="E14" s="28">
         <v>10</v>
       </c>
-      <c r="F14" s="56" t="s">
-        <v>70</v>
-      </c>
-      <c r="G14" s="57">
+      <c r="F14" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="G14" s="19">
         <v>613</v>
       </c>
-      <c r="H14" s="67">
+      <c r="H14" s="28">
         <f t="shared" si="0"/>
         <v>6130</v>
       </c>
-      <c r="I14" s="67">
+      <c r="I14" s="28">
         <f>SUM(H10:H14)</f>
         <v>11454.25</v>
       </c>
     </row>
     <row r="15" spans="2:11" ht="30">
-      <c r="E15" s="66"/>
-      <c r="G15" s="62" t="s">
-        <v>71</v>
-      </c>
-      <c r="H15" s="67"/>
-      <c r="I15" s="67">
+      <c r="E15" s="27"/>
+      <c r="G15" s="23" t="s">
+        <v>63</v>
+      </c>
+      <c r="H15" s="28"/>
+      <c r="I15" s="28">
         <f>I14*0.15</f>
         <v>1718.1375</v>
       </c>
     </row>
-    <row r="16" spans="2:11" ht="16.8">
-      <c r="G16" s="63" t="s">
-        <v>72</v>
-      </c>
-      <c r="I16" s="67">
+    <row r="16" spans="2:11" ht="16.5">
+      <c r="G16" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="I16" s="28">
         <f>SUM(I9:I15)</f>
         <v>26562.387500000001</v>
       </c>
     </row>
-    <row r="17" spans="3:9" ht="16.8">
-      <c r="C17" s="47" t="s">
-        <v>73</v>
-      </c>
-      <c r="G17" s="63" t="s">
-        <v>74</v>
-      </c>
-      <c r="I17" s="67">
+    <row r="17" spans="3:9" ht="16.5">
+      <c r="C17" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="G17" s="24" t="s">
+        <v>66</v>
+      </c>
+      <c r="I17" s="28">
         <f>FLOOR(I16*0.15,0.01)</f>
         <v>3984.35</v>
       </c>
     </row>
-    <row r="18" spans="3:9" ht="18">
-      <c r="C18" s="64">
+    <row r="18" spans="3:9" ht="16.5">
+      <c r="C18" s="25">
         <f>+I18</f>
         <v>30546.737499999999</v>
       </c>
-      <c r="D18" s="49" t="s">
-        <v>75</v>
-      </c>
-      <c r="E18" s="67">
+      <c r="D18" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="E18" s="28">
         <f>FLOOR(C18/C19,0.01)</f>
         <v>3054.67</v>
       </c>
-      <c r="F18" s="47" t="s">
-        <v>76</v>
-      </c>
-      <c r="G18" s="63" t="s">
-        <v>77</v>
-      </c>
-      <c r="I18" s="67">
+      <c r="F18" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="G18" s="24" t="s">
+        <v>69</v>
+      </c>
+      <c r="I18" s="28">
         <f>SUM(I16:I17)</f>
         <v>30546.737499999999</v>
       </c>
     </row>
     <row r="19" spans="3:9">
-      <c r="C19" s="65">
+      <c r="C19" s="26">
         <v>10</v>
       </c>
-      <c r="E19" s="67"/>
-      <c r="I19" s="67"/>
+      <c r="E19" s="28"/>
+      <c r="I19" s="28"/>
     </row>
     <row r="20" spans="3:9">
-      <c r="I20" s="67"/>
+      <c r="I20" s="28"/>
     </row>
   </sheetData>
   <mergeCells count="7">

</xml_diff>

<commit_message>
little changes to laganshil and given again
</commit_message>
<xml_diff>
--- a/बजेट माग estimate/lagansil krishak samuha.xlsx
+++ b/बजेट माग estimate/lagansil krishak samuha.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4BC52F6-C133-4B16-AAC9-3969749A9F55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B624D2AB-536A-4D77-992A-026EC713474C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -574,22 +574,22 @@
     <t>Length (m)</t>
   </si>
   <si>
-    <t>-Fabrication of chain link mesh size 3"x3" 10 gauge</t>
-  </si>
-  <si>
     <t>-Skilled   mason</t>
   </si>
   <si>
     <t>-Unskilled mason</t>
   </si>
   <si>
-    <t>-Vertical pole (40x40x2)</t>
-  </si>
-  <si>
     <t>Estimated Sheet</t>
   </si>
   <si>
     <t xml:space="preserve">Date:                </t>
+  </si>
+  <si>
+    <t>-Fabrication of chain link mesh size 4"x4" 10 gauge</t>
+  </si>
+  <si>
+    <t>-Vertical pole equal angle size (40x40x3)</t>
   </si>
 </sst>
 </file>
@@ -1092,6 +1092,24 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1107,19 +1125,6 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1141,11 +1146,6 @@
     <xf numFmtId="0" fontId="21" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -1761,68 +1761,68 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="15.75">
-      <c r="A1" s="73" t="s">
+      <c r="A1" s="70" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="73"/>
-      <c r="C1" s="73"/>
-      <c r="D1" s="73"/>
-      <c r="E1" s="73"/>
-      <c r="F1" s="73"/>
-      <c r="G1" s="73"/>
-      <c r="H1" s="73"/>
-      <c r="I1" s="73"/>
-      <c r="J1" s="73"/>
-      <c r="K1" s="73"/>
-      <c r="L1" s="73"/>
+      <c r="B1" s="70"/>
+      <c r="C1" s="70"/>
+      <c r="D1" s="70"/>
+      <c r="E1" s="70"/>
+      <c r="F1" s="70"/>
+      <c r="G1" s="70"/>
+      <c r="H1" s="70"/>
+      <c r="I1" s="70"/>
+      <c r="J1" s="70"/>
+      <c r="K1" s="70"/>
+      <c r="L1" s="70"/>
     </row>
     <row r="2" spans="1:12" ht="20.25">
-      <c r="A2" s="74" t="s">
+      <c r="A2" s="71" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="74"/>
-      <c r="C2" s="74"/>
-      <c r="D2" s="74"/>
-      <c r="E2" s="74"/>
-      <c r="F2" s="74"/>
-      <c r="G2" s="74"/>
-      <c r="H2" s="74"/>
-      <c r="I2" s="74"/>
-      <c r="J2" s="74"/>
-      <c r="K2" s="74"/>
-      <c r="L2" s="74"/>
+      <c r="B2" s="71"/>
+      <c r="C2" s="71"/>
+      <c r="D2" s="71"/>
+      <c r="E2" s="71"/>
+      <c r="F2" s="71"/>
+      <c r="G2" s="71"/>
+      <c r="H2" s="71"/>
+      <c r="I2" s="71"/>
+      <c r="J2" s="71"/>
+      <c r="K2" s="71"/>
+      <c r="L2" s="71"/>
     </row>
     <row r="3" spans="1:12" ht="15.75">
-      <c r="A3" s="73" t="s">
+      <c r="A3" s="70" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="73"/>
-      <c r="C3" s="73"/>
-      <c r="D3" s="73"/>
-      <c r="E3" s="73"/>
-      <c r="F3" s="73"/>
-      <c r="G3" s="73"/>
-      <c r="H3" s="73"/>
-      <c r="I3" s="73"/>
-      <c r="J3" s="73"/>
-      <c r="K3" s="73"/>
-      <c r="L3" s="73"/>
+      <c r="B3" s="70"/>
+      <c r="C3" s="70"/>
+      <c r="D3" s="70"/>
+      <c r="E3" s="70"/>
+      <c r="F3" s="70"/>
+      <c r="G3" s="70"/>
+      <c r="H3" s="70"/>
+      <c r="I3" s="70"/>
+      <c r="J3" s="70"/>
+      <c r="K3" s="70"/>
+      <c r="L3" s="70"/>
     </row>
     <row r="4" spans="1:12" ht="15.75">
-      <c r="A4" s="83" t="s">
-        <v>83</v>
-      </c>
-      <c r="B4" s="83"/>
-      <c r="C4" s="83"/>
-      <c r="D4" s="83"/>
-      <c r="E4" s="83"/>
-      <c r="F4" s="83"/>
-      <c r="G4" s="83"/>
-      <c r="H4" s="83"/>
-      <c r="I4" s="83"/>
-      <c r="J4" s="83"/>
-      <c r="K4" s="83"/>
-      <c r="L4" s="83"/>
+      <c r="A4" s="72" t="s">
+        <v>81</v>
+      </c>
+      <c r="B4" s="72"/>
+      <c r="C4" s="72"/>
+      <c r="D4" s="72"/>
+      <c r="E4" s="72"/>
+      <c r="F4" s="72"/>
+      <c r="G4" s="72"/>
+      <c r="H4" s="72"/>
+      <c r="I4" s="72"/>
+      <c r="J4" s="72"/>
+      <c r="K4" s="72"/>
+      <c r="L4" s="72"/>
     </row>
     <row r="5" spans="1:12" ht="16.5">
       <c r="A5" s="65"/>
@@ -1854,26 +1854,26 @@
       <c r="I6" s="4"/>
       <c r="J6" s="5"/>
       <c r="K6" s="4"/>
-      <c r="L6" s="84" t="s">
+      <c r="L6" s="66" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="16.5">
       <c r="A7" s="4"/>
-      <c r="B7" s="75" t="s">
+      <c r="B7" s="73" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="75"/>
-      <c r="D7" s="75"/>
-      <c r="E7" s="75"/>
-      <c r="F7" s="75"/>
-      <c r="G7" s="75"/>
+      <c r="C7" s="73"/>
+      <c r="D7" s="73"/>
+      <c r="E7" s="73"/>
+      <c r="F7" s="73"/>
+      <c r="G7" s="73"/>
       <c r="H7" s="6"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
-      <c r="L7" s="85" t="s">
-        <v>84</v>
+      <c r="L7" s="67" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="15.75">
@@ -1920,8 +1920,8 @@
         <v>19</v>
       </c>
       <c r="D9" s="47">
-        <f>ROUNDUP(400/3,0)+1</f>
-        <v>135</v>
+        <f>ROUNDUP(400/2.3,0)+1</f>
+        <v>175</v>
       </c>
       <c r="E9" s="47">
         <v>0.45</v>
@@ -1934,7 +1934,7 @@
       </c>
       <c r="H9" s="47">
         <f>D9*E9*F9*G9</f>
-        <v>16.4025</v>
+        <v>21.262499999999999</v>
       </c>
       <c r="I9" s="48" t="s">
         <v>6</v>
@@ -1944,7 +1944,7 @@
       </c>
       <c r="K9" s="47">
         <f>H9*J9</f>
-        <v>11057.2533</v>
+        <v>14333.476499999999</v>
       </c>
       <c r="L9" s="49"/>
     </row>
@@ -1970,7 +1970,7 @@
       </c>
       <c r="D11" s="51">
         <f>D9</f>
-        <v>135</v>
+        <v>175</v>
       </c>
       <c r="E11" s="51">
         <v>0.3</v>
@@ -1983,7 +1983,7 @@
       </c>
       <c r="H11" s="51">
         <f>D11*E11*F11*G11</f>
-        <v>5.4675000000000002</v>
+        <v>7.0875000000000004</v>
       </c>
       <c r="I11" s="51" t="s">
         <v>6</v>
@@ -1993,7 +1993,7 @@
       </c>
       <c r="K11" s="51">
         <f>J11*H11</f>
-        <v>72997.139250000007</v>
+        <v>94625.921250000014</v>
       </c>
       <c r="L11" s="49"/>
     </row>
@@ -2011,7 +2011,7 @@
       <c r="J12" s="51"/>
       <c r="K12" s="51">
         <f>0.13*H11*4169.92</f>
-        <v>2963.8748880000003</v>
+        <v>3842.0600400000003</v>
       </c>
       <c r="L12" s="49"/>
     </row>
@@ -2029,7 +2029,7 @@
       <c r="J13" s="53"/>
       <c r="K13" s="51">
         <f>0.13*H11*1414.16</f>
-        <v>1005.1495740000001</v>
+        <v>1302.9716700000001</v>
       </c>
       <c r="L13" s="49"/>
     </row>
@@ -2047,7 +2047,7 @@
       <c r="J14" s="53"/>
       <c r="K14" s="51">
         <f>0.13*H11*(1652.5+737.97+349.56)</f>
-        <v>1947.5448232500003</v>
+        <v>2524.5951412500003</v>
       </c>
       <c r="L14" s="49"/>
     </row>
@@ -2147,14 +2147,14 @@
       <c r="K19" s="51"/>
       <c r="L19" s="49"/>
     </row>
-    <row r="20" spans="1:15" ht="15.75">
+    <row r="20" spans="1:15" ht="31.5">
       <c r="B20" s="49"/>
-      <c r="C20" s="61" t="s">
-        <v>82</v>
+      <c r="C20" s="60" t="s">
+        <v>84</v>
       </c>
       <c r="D20" s="51">
         <f>D11</f>
-        <v>135</v>
+        <v>175</v>
       </c>
       <c r="E20" s="51">
         <f>6.5/3.28</f>
@@ -2162,11 +2162,11 @@
       </c>
       <c r="F20" s="51"/>
       <c r="G20" s="51">
-        <v>1.19</v>
+        <v>1.75</v>
       </c>
       <c r="H20" s="51">
         <f>D20*E20*G20</f>
-        <v>318.36128048780489</v>
+        <v>606.89786585365857</v>
       </c>
       <c r="I20" s="51" t="s">
         <v>26</v>
@@ -2176,7 +2176,7 @@
       </c>
       <c r="K20" s="51">
         <f>H20*J20</f>
-        <v>29607.599085365855</v>
+        <v>56441.501524390245</v>
       </c>
       <c r="L20" s="49"/>
     </row>
@@ -2194,14 +2194,14 @@
       <c r="J21" s="51"/>
       <c r="K21" s="51">
         <f>0.13*K20</f>
-        <v>3848.9878810975611</v>
+        <v>7337.3951981707323</v>
       </c>
       <c r="L21" s="49"/>
     </row>
     <row r="22" spans="1:15" ht="31.5">
       <c r="B22" s="49"/>
       <c r="C22" s="60" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D22" s="51">
         <v>1</v>
@@ -2222,11 +2222,11 @@
         <v>5</v>
       </c>
       <c r="J22" s="51">
-        <v>501</v>
+        <v>399</v>
       </c>
       <c r="K22" s="51">
         <f>H22*J22</f>
-        <v>274855.22706491925</v>
+        <v>218896.67784212131</v>
       </c>
       <c r="L22" s="49"/>
     </row>
@@ -2244,7 +2244,7 @@
       <c r="J23" s="49"/>
       <c r="K23" s="51">
         <f>0.13*K22</f>
-        <v>35731.179518439501</v>
+        <v>28456.568119475771</v>
       </c>
       <c r="L23" s="49"/>
     </row>
@@ -2267,17 +2267,17 @@
     <row r="25" spans="1:15" ht="15.75">
       <c r="B25" s="49"/>
       <c r="C25" s="61" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D25" s="57">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E25" s="49"/>
       <c r="F25" s="49"/>
       <c r="G25" s="49"/>
       <c r="H25" s="51">
         <f>D25</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I25" s="51" t="s">
         <v>28</v>
@@ -2287,7 +2287,7 @@
       </c>
       <c r="K25" s="51">
         <f>H25*J25</f>
-        <v>5175</v>
+        <v>6210</v>
       </c>
       <c r="L25" s="49"/>
       <c r="O25" s="8" t="s">
@@ -2297,17 +2297,17 @@
     <row r="26" spans="1:15" ht="15.75">
       <c r="B26" s="49"/>
       <c r="C26" s="61" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D26" s="57">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E26" s="49"/>
       <c r="F26" s="49"/>
       <c r="G26" s="49"/>
       <c r="H26" s="51">
         <f>D26</f>
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="I26" s="51" t="s">
         <v>28</v>
@@ -2317,7 +2317,7 @@
       </c>
       <c r="K26" s="51">
         <f>H26*J26</f>
-        <v>12375</v>
+        <v>14850</v>
       </c>
       <c r="L26" s="49"/>
       <c r="O26" s="8" t="s">
@@ -2396,7 +2396,7 @@
       <c r="J30" s="49"/>
       <c r="K30" s="59">
         <f>SUM(K9:K28)</f>
-        <v>486547.86818507221</v>
+        <v>483805.08008540812</v>
       </c>
       <c r="L30" s="49"/>
     </row>
@@ -2405,11 +2405,11 @@
       <c r="C32" s="32" t="s">
         <v>71</v>
       </c>
-      <c r="D32" s="66">
+      <c r="D32" s="74">
         <f>K30</f>
-        <v>486547.86818507221</v>
-      </c>
-      <c r="E32" s="66"/>
+        <v>483805.08008540812</v>
+      </c>
+      <c r="E32" s="74"/>
       <c r="F32" s="64"/>
       <c r="G32" s="34"/>
       <c r="H32" s="31"/>
@@ -2421,24 +2421,24 @@
       <c r="C33" s="62" t="s">
         <v>72</v>
       </c>
-      <c r="D33" s="67">
+      <c r="D33" s="75">
         <v>480000</v>
       </c>
-      <c r="E33" s="68"/>
+      <c r="E33" s="76"/>
       <c r="F33" s="63"/>
     </row>
     <row r="34" spans="3:9" hidden="1">
       <c r="C34" s="32" t="s">
         <v>73</v>
       </c>
-      <c r="D34" s="69">
+      <c r="D34" s="77">
         <f>D33-D36-D37</f>
         <v>456000</v>
       </c>
-      <c r="E34" s="70"/>
+      <c r="E34" s="78"/>
       <c r="F34" s="33">
         <f>D34/D32*100</f>
-        <v>93.721508163416217</v>
+        <v>94.252834203291215</v>
       </c>
       <c r="G34" s="28"/>
     </row>
@@ -2446,25 +2446,25 @@
       <c r="C35" s="32" t="s">
         <v>74</v>
       </c>
-      <c r="D35" s="66">
+      <c r="D35" s="74">
         <f>D32-D34</f>
-        <v>30547.868185072206</v>
-      </c>
-      <c r="E35" s="66"/>
+        <v>27805.080085408117</v>
+      </c>
+      <c r="E35" s="74"/>
       <c r="F35" s="33">
         <f>100-F34</f>
-        <v>6.2784918365837825</v>
+        <v>5.747165796708785</v>
       </c>
     </row>
     <row r="36" spans="3:9" hidden="1">
       <c r="C36" s="32" t="s">
         <v>75</v>
       </c>
-      <c r="D36" s="71">
+      <c r="D36" s="68">
         <f>D33*0.03</f>
         <v>14400</v>
       </c>
-      <c r="E36" s="72"/>
+      <c r="E36" s="69"/>
       <c r="F36" s="33">
         <v>0</v>
       </c>
@@ -2473,11 +2473,11 @@
       <c r="C37" s="32" t="s">
         <v>76</v>
       </c>
-      <c r="D37" s="71">
+      <c r="D37" s="68">
         <f>D33*0.02</f>
         <v>9600</v>
       </c>
-      <c r="E37" s="72"/>
+      <c r="E37" s="69"/>
       <c r="F37" s="33">
         <v>0</v>
       </c>
@@ -2589,15 +2589,15 @@
       <c r="B2" s="9">
         <v>297</v>
       </c>
-      <c r="C2" s="79" t="s">
+      <c r="C2" s="82" t="s">
         <v>38</v>
       </c>
-      <c r="D2" s="80"/>
-      <c r="E2" s="80"/>
-      <c r="F2" s="80"/>
-      <c r="G2" s="80"/>
-      <c r="H2" s="80"/>
-      <c r="I2" s="80"/>
+      <c r="D2" s="83"/>
+      <c r="E2" s="83"/>
+      <c r="F2" s="83"/>
+      <c r="G2" s="83"/>
+      <c r="H2" s="83"/>
+      <c r="I2" s="83"/>
       <c r="J2" s="29"/>
       <c r="K2" s="29"/>
     </row>
@@ -2605,48 +2605,48 @@
       <c r="B3" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="C3" s="81" t="s">
+      <c r="C3" s="84" t="s">
         <v>40</v>
       </c>
-      <c r="D3" s="80"/>
-      <c r="E3" s="80"/>
-      <c r="F3" s="80"/>
-      <c r="G3" s="80"/>
-      <c r="H3" s="80"/>
-      <c r="I3" s="80"/>
+      <c r="D3" s="83"/>
+      <c r="E3" s="83"/>
+      <c r="F3" s="83"/>
+      <c r="G3" s="83"/>
+      <c r="H3" s="83"/>
+      <c r="I3" s="83"/>
     </row>
     <row r="4" spans="2:11">
-      <c r="C4" s="80" t="s">
+      <c r="C4" s="83" t="s">
         <v>41</v>
       </c>
-      <c r="D4" s="80"/>
-      <c r="E4" s="80"/>
-      <c r="F4" s="80"/>
-      <c r="G4" s="80"/>
-      <c r="H4" s="80"/>
-      <c r="I4" s="80"/>
+      <c r="D4" s="83"/>
+      <c r="E4" s="83"/>
+      <c r="F4" s="83"/>
+      <c r="G4" s="83"/>
+      <c r="H4" s="83"/>
+      <c r="I4" s="83"/>
     </row>
     <row r="5" spans="2:11">
-      <c r="C5" s="80" t="s">
+      <c r="C5" s="83" t="s">
         <v>42</v>
       </c>
-      <c r="D5" s="80"/>
-      <c r="E5" s="80"/>
-      <c r="F5" s="80"/>
-      <c r="G5" s="80"/>
-      <c r="H5" s="80"/>
-      <c r="I5" s="80"/>
+      <c r="D5" s="83"/>
+      <c r="E5" s="83"/>
+      <c r="F5" s="83"/>
+      <c r="G5" s="83"/>
+      <c r="H5" s="83"/>
+      <c r="I5" s="83"/>
     </row>
     <row r="6" spans="2:11">
-      <c r="C6" s="82" t="s">
+      <c r="C6" s="85" t="s">
         <v>43</v>
       </c>
-      <c r="D6" s="82"/>
-      <c r="E6" s="82"/>
-      <c r="F6" s="82"/>
-      <c r="G6" s="82"/>
-      <c r="H6" s="82"/>
-      <c r="I6" s="82"/>
+      <c r="D6" s="85"/>
+      <c r="E6" s="85"/>
+      <c r="F6" s="85"/>
+      <c r="G6" s="85"/>
+      <c r="H6" s="85"/>
+      <c r="I6" s="85"/>
     </row>
     <row r="7" spans="2:11" ht="63">
       <c r="C7" s="12" t="s">
@@ -2672,7 +2672,7 @@
       </c>
     </row>
     <row r="8" spans="2:11" ht="16.5">
-      <c r="C8" s="76" t="s">
+      <c r="C8" s="79" t="s">
         <v>51</v>
       </c>
       <c r="D8" s="14" t="s">
@@ -2694,7 +2694,7 @@
       <c r="I8" s="28"/>
     </row>
     <row r="9" spans="2:11" ht="16.5">
-      <c r="C9" s="78"/>
+      <c r="C9" s="81"/>
       <c r="D9" s="17" t="s">
         <v>54</v>
       </c>
@@ -2717,7 +2717,7 @@
       </c>
     </row>
     <row r="10" spans="2:11" ht="16.5">
-      <c r="C10" s="76" t="s">
+      <c r="C10" s="79" t="s">
         <v>55</v>
       </c>
       <c r="D10" s="14" t="s">
@@ -2740,7 +2740,7 @@
       <c r="I10" s="28"/>
     </row>
     <row r="11" spans="2:11" ht="16.5">
-      <c r="C11" s="77"/>
+      <c r="C11" s="80"/>
       <c r="D11" s="20" t="s">
         <v>58</v>
       </c>
@@ -2760,7 +2760,7 @@
       <c r="I11" s="28"/>
     </row>
     <row r="12" spans="2:11" ht="16.5">
-      <c r="C12" s="77"/>
+      <c r="C12" s="80"/>
       <c r="D12" s="20" t="s">
         <v>59</v>
       </c>
@@ -2780,7 +2780,7 @@
       <c r="I12" s="28"/>
     </row>
     <row r="13" spans="2:11" ht="28.5">
-      <c r="C13" s="77"/>
+      <c r="C13" s="80"/>
       <c r="D13" s="22" t="s">
         <v>60</v>
       </c>
@@ -2801,7 +2801,7 @@
       <c r="I13" s="28"/>
     </row>
     <row r="14" spans="2:11" ht="28.5">
-      <c r="C14" s="78"/>
+      <c r="C14" s="81"/>
       <c r="D14" s="22" t="s">
         <v>61</v>
       </c>

</xml_diff>